<commit_message>
feat: Add multi-SKU tree JSON harvesting, multi-line Excel generation, metadata retention, and 100% test coverage
</commit_message>
<xml_diff>
--- a/output/product_spec.xlsx
+++ b/output/product_spec.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Product Overview &amp; IDs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Full Specifications" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Multi-SKU Catalog &amp; IDs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,12 +51,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00C00000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00008000"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -101,19 +94,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -479,18 +469,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>UNIVERSAL PRODUCT SPECIFICATION SHEET</t>
+          <t>UNIVERSAL PRODUCT INTELLIGENCE - MULTI-SKU SPECIFICATION SHEET</t>
         </is>
       </c>
     </row>
@@ -498,12 +498,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Product Title:</t>
+          <t>Product Family:</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Incomplete Product</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>TechCorp</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -534,196 +534,163 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Price / Currency:</t>
+          <t>Confidence Score:</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>N/A USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp:</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Identifier Type</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Data Sources:</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>SKU ID</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Variant Name</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>GTIN-14</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>UPC-12</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>EAN-13</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>MPN</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>VPN</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>ASIN</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>UNSPSC</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>HS Code</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Attributes &amp; Specifications</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>GTIN-14</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>UPC-12</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>MISSING</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>EAN-13</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>MPN / VPN</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>ASIN</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>UNSPSC Code</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>HS Code</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>ISBN</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>978-3-16-148410-0</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>Attribute Name</t>
-        </is>
-      </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>Attribute Value</t>
+          <t>NO-ID-SKU</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr"/>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>MISSING IDs</t>
         </is>
       </c>
     </row>

</xml_diff>